<commit_message>
Updated the backlog and task distribution for case closing and staff changes
</commit_message>
<xml_diff>
--- a/docs/product-backlog.xlsx
+++ b/docs/product-backlog.xlsx
@@ -1470,7 +1470,7 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>As a Finance Officer, I want to edit disputed pending charges, void incorrect invoices, and refund paid charges, so that billing errors can be corrected at any stage.</t>
+          <t>As a Finance Officer, I want to edit disputed pending charges, void incorrect invoices, and refund paid charges, so that billing errors can be corrected while the case is open.</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
@@ -1502,7 +1502,7 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>As an Associate, I want to close an active case with a final resolution status, so that completed cases are officially closed.</t>
+          <t>As an Associate, I want to close an active case with a final resolution status, so that completed cases are officially closed once all of their billing is settled.</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
@@ -1534,7 +1534,7 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>As a Partner, I want to reassign the Associate or Paralegal on a consultation or case, so that staffing can be corrected after the fact.</t>
+          <t>As a Partner, I want to reassign the Associate or Paralegal on a consultation before its case is opened or on an open case, so that staffing can be corrected after the fact.</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Updated the backlog and task distribution for the consultation request rename
</commit_message>
<xml_diff>
--- a/docs/product-backlog.xlsx
+++ b/docs/product-backlog.xlsx
@@ -768,7 +768,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>As a Client, I want to submit a consultation request with legal issue details and track its status and consultation meeting, so that the firm can evaluate my legal matter and I know where it stands.</t>
+          <t>As a Client, I want to request a consultation with legal issue details and track its status and consultation meeting, so that the firm can evaluate my legal matter and I know where it stands.</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -1598,7 +1598,7 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>As a Client Relations Officer, I want to submit walk-in clients' consultation requests and follow them and their scheduled consultation meetings, so that a Partner can perform a conflict check.</t>
+          <t>As a Client Relations Officer, I want to request consultations for walk-in clients and follow them and their scheduled consultation meetings, so that a Partner can perform a conflict check.</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">

</xml_diff>